<commit_message>
feat: Requisição com parâmetro (AvailabilitySlot)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +588,482 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14:06:30</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>22180</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>79.31</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Home</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14:09:50</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>14:09:50</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>79.97</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:09:53</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>84.77</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>84.89</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:10:04</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>85.02</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:15:24</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>22992</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>83.18000000000001</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:21:07</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>24019</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>83.34</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:27:10</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>24392</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>83.04000000000001</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:27:26</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>24418</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>83.13</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:30:30</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>24712</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>79.97</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14:31:36</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>24784</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:31:40</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>24784</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>83.27</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:31:46</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>24784</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>83.52</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:37:42</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>25203</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>83.22</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:38:10</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>25203</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>83.59</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:40:10</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>25401</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>83.53</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Inserção de mensagem (LOGS)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1064,6 +1064,258 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>25975</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>79.79000000000001</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:46:48</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>26043</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:48:08</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>26109</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>80.06999999999999</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:49:42</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>26223</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>80.17</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:53:36</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>26750</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>83.02</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:53:47</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>26750</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:58:14</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>27311</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>83.38</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:58:17</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>27311</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>83.76000000000001</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:00:39</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>27492</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Resolução do problema 'ColumnElement[bool]'
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1316,6 +1316,174 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>18:54:00</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>76731</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>83.47</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:11:10</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>78986</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>83.89</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:26:21</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>81269</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>86.97</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>81830</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>87.20999999999999</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:29:55</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>81830</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>87.45999999999999</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:32:20</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>82295</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: Reestruturação dos Models
- Mapped[Type] e mapped_column
- user.py e sessions.py
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1484,6 +1484,286 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:36:55</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>83952</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>85.11</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:37:23</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>84026</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>19:41:45</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>84.97</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:41:51</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>85.47</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:41:56</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>86.65000000000001</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:42:01</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:42:10</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:43:09</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>87.28</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>19:43:13</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:43:20</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>84806</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Leitura para as Línguas (Idiomas)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1764,6 +1764,34 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:00:27</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>87374</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>85.51000000000001</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Languages</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Leitura para as Tecnologias
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-02.xlsx
+++ b/api/desempenho/2025-07-02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1792,6 +1792,34 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:08:05</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>88274</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>86.06999999999999</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Acesso na rota Tech Stacks</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>